<commit_message>
Update RangeSayacv3.xlsx with new theme data
</commit_message>
<xml_diff>
--- a/RangeSayacv3.xlsx
+++ b/RangeSayacv3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaank\Downloads\IpekyolRangeSayac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A5928DD-5722-4621-9FE0-EF49A9D6F685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C705DD9-B55C-499E-AD24-F0DBBAC86C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BF37BD-FBCE-455B-B84F-487EBCBBCEE9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>P_Opt</t>
   </si>
@@ -47,27 +47,101 @@
     <t>Tema_Id</t>
   </si>
   <si>
-    <t>SS26_WORKSHOP_B_TEMA_1</t>
-  </si>
-  <si>
-    <t>SS26_WORKSHOP_TEMA_3</t>
-  </si>
-  <si>
-    <t>SS26_WORKSHOP_TEMA_2</t>
-  </si>
-  <si>
-    <t>SS26_WORKSHOP_TEMA_1</t>
+    <t>TWS-TEMA 1</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 2</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 3</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 4</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 5</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 6</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 7</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 8</t>
+  </si>
+  <si>
+    <t>TWS-TEMA 9</t>
+  </si>
+  <si>
+    <t>B-MONO 1</t>
+  </si>
+  <si>
+    <t>B-MONO 2</t>
+  </si>
+  <si>
+    <t>B-MONO 3</t>
+  </si>
+  <si>
+    <t>B-SCT1</t>
+  </si>
+  <si>
+    <t>B-SCT2</t>
+  </si>
+  <si>
+    <t>B-SCT3</t>
+  </si>
+  <si>
+    <t>B-SCT4</t>
+  </si>
+  <si>
+    <t>B-SCT5</t>
+  </si>
+  <si>
+    <t>B-BCT1</t>
+  </si>
+  <si>
+    <t>B-SCT6</t>
+  </si>
+  <si>
+    <t>MONO-SCT1</t>
+  </si>
+  <si>
+    <t>MONO-SCT2</t>
+  </si>
+  <si>
+    <t>MONO-SCT3</t>
+  </si>
+  <si>
+    <t>B-JEAN P1-IPK</t>
+  </si>
+  <si>
+    <t>MONO-SCT4</t>
+  </si>
+  <si>
+    <t>MONO-SCT5</t>
+  </si>
+  <si>
+    <t>MONO-SCT6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -77,8 +151,15 @@
       <family val="2"/>
       <charset val="162"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="162"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -91,8 +172,32 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEFAD2"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -109,16 +214,65 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="9" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{F63E26E7-0016-4D30-9356-C85115199214}"/>
+    <cellStyle name="Normal 3" xfId="1" xr:uid="{909B3FE4-1AD4-421E-8DAF-8F839728EA5B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -450,7 +604,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F8E911-A934-46A7-9C01-3A6D45D6A799}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
@@ -469,47 +623,289 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
-        <v>1032</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="3">
+        <v>1079</v>
+      </c>
+      <c r="C2" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="5">
+        <v>1080</v>
+      </c>
+      <c r="C3" s="4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1087</v>
+      </c>
+      <c r="C4" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="5">
+        <v>1092</v>
+      </c>
+      <c r="C5" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1098</v>
+      </c>
+      <c r="C6" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="5">
+        <v>1099</v>
+      </c>
+      <c r="C7" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="3">
+        <v>1106</v>
+      </c>
+      <c r="C8" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5">
+        <v>1110</v>
+      </c>
+      <c r="C9" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3">
+        <v>1116</v>
+      </c>
+      <c r="C10" s="4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="5">
+        <v>1086</v>
+      </c>
+      <c r="C11" s="8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="3">
+        <v>1105</v>
+      </c>
+      <c r="C12" s="8">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="5">
+        <v>1115</v>
+      </c>
+      <c r="C13" s="7">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="5">
+        <v>1076</v>
+      </c>
+      <c r="C14" s="11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="5">
+        <v>1083</v>
+      </c>
+      <c r="C15" s="11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="5">
+        <v>1089</v>
+      </c>
+      <c r="C16" s="11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="5">
+        <v>1095</v>
+      </c>
+      <c r="C17" s="11">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="5">
+        <v>1102</v>
+      </c>
+      <c r="C18" s="11">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="5">
+        <v>1112</v>
+      </c>
+      <c r="C19" s="11">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" s="10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>1031</v>
-      </c>
-      <c r="C3">
+      <c r="B20" s="5">
+        <v>1108</v>
+      </c>
+      <c r="C20" s="12">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>1030</v>
-      </c>
-      <c r="C4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="3">
+        <v>1077</v>
+      </c>
+      <c r="C21" s="14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="3">
+        <v>1084</v>
+      </c>
+      <c r="C22" s="14">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>1029</v>
-      </c>
-      <c r="C5">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="3">
+        <v>1090</v>
+      </c>
+      <c r="C23" s="14">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="13" t="s">
         <v>25</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1094</v>
+      </c>
+      <c r="C24" s="14">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="3">
+        <v>1096</v>
+      </c>
+      <c r="C25" s="14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="3">
+        <v>1103</v>
+      </c>
+      <c r="C26" s="14">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="3">
+        <v>1113</v>
+      </c>
+      <c r="C27" s="14">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Ensure 1-to-1 placeholder to colorway matching in range-count-source
</commit_message>
<xml_diff>
--- a/RangeSayacv3.xlsx
+++ b/RangeSayacv3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaank\Downloads\IpekyolRangeSayac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C705DD9-B55C-499E-AD24-F0DBBAC86C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078DA04F-EA18-448C-B950-27D77FE045EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F6BF37BD-FBCE-455B-B84F-487EBCBBCEE9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="32">
   <si>
     <t>P_Opt</t>
   </si>
@@ -123,6 +123,15 @@
   </si>
   <si>
     <t>MONO-SCT6</t>
+  </si>
+  <si>
+    <t>Marka</t>
+  </si>
+  <si>
+    <t>TWIST</t>
+  </si>
+  <si>
+    <t>IPEKYOL</t>
   </si>
 </sst>
 </file>
@@ -242,7 +251,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -262,12 +271,7 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,307 +608,389 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F8E911-A934-46A7-9C01-3A6D45D6A799}">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="3">
         <v>1079</v>
       </c>
-      <c r="C2" s="4">
+      <c r="D2" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="5">
         <v>1080</v>
       </c>
-      <c r="C3" s="4">
+      <c r="D3" s="4">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="3">
         <v>1087</v>
       </c>
-      <c r="C4" s="4">
+      <c r="D4" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="5">
         <v>1092</v>
       </c>
-      <c r="C5" s="4">
+      <c r="D5" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="3">
         <v>1098</v>
       </c>
-      <c r="C6" s="4">
+      <c r="D6" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="5">
         <v>1099</v>
       </c>
-      <c r="C7" s="4">
+      <c r="D7" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="3">
         <v>1106</v>
       </c>
-      <c r="C8" s="4">
+      <c r="D8" s="4">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="5">
         <v>1110</v>
       </c>
-      <c r="C9" s="4">
+      <c r="D9" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="3">
         <v>1116</v>
       </c>
-      <c r="C10" s="4">
+      <c r="D10" s="4">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="5">
         <v>1086</v>
       </c>
-      <c r="C11" s="8">
+      <c r="D11" s="8">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="3">
         <v>1105</v>
       </c>
-      <c r="C12" s="8">
+      <c r="D12" s="8">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="5">
         <v>1115</v>
       </c>
-      <c r="C13" s="7">
+      <c r="D13" s="7">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="5">
         <v>1076</v>
       </c>
-      <c r="C14" s="11">
+      <c r="D14" s="4">
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="5">
         <v>1083</v>
       </c>
-      <c r="C15" s="11">
+      <c r="D15" s="4">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="5">
         <v>1089</v>
       </c>
-      <c r="C16" s="11">
+      <c r="D16" s="4">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="5">
         <v>1095</v>
       </c>
-      <c r="C17" s="11">
+      <c r="D17" s="4">
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="5">
         <v>1102</v>
       </c>
-      <c r="C18" s="11">
+      <c r="D18" s="4">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="5">
         <v>1112</v>
       </c>
-      <c r="C19" s="11">
+      <c r="D19" s="4">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="5">
         <v>1108</v>
       </c>
-      <c r="C20" s="12">
+      <c r="D20" s="11">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="13" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="3">
         <v>1077</v>
       </c>
-      <c r="C21" s="14">
+      <c r="D21" s="8">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="3">
         <v>1084</v>
       </c>
-      <c r="C22" s="14">
+      <c r="D22" s="8">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="3">
         <v>1090</v>
       </c>
-      <c r="C23" s="14">
+      <c r="D23" s="8">
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C24" s="3">
         <v>1094</v>
       </c>
-      <c r="C24" s="14">
+      <c r="D24" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B25" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="3">
         <v>1096</v>
       </c>
-      <c r="C25" s="14">
+      <c r="D25" s="8">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="3">
+      <c r="B26" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C26" s="3">
         <v>1103</v>
       </c>
-      <c r="C26" s="14">
+      <c r="D26" s="8">
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" s="13" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B27" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="3">
         <v>1113</v>
       </c>
-      <c r="C27" s="14">
+      <c r="D27" s="8">
         <v>20</v>
       </c>
     </row>

</xml_diff>